<commit_message>
Added all l2 controls to SQL
</commit_message>
<xml_diff>
--- a/02_WorkingDocs/CMMCFledge_Workbook.xlsx
+++ b/02_WorkingDocs/CMMCFledge_Workbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ckm32\OneDrive\Desktop\CMMCFledge\02_WorkingDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8D53A8F-76B9-42C2-A2A1-9B6CB0B3E253}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86802CD0-1F78-494F-90BC-5C846163625D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="40905" yWindow="4980" windowWidth="23040" windowHeight="12120" activeTab="1" xr2:uid="{208106DA-3D21-4604-99AA-9AD5A5B6DE72}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="87">
   <si>
     <t>Week:</t>
   </si>
@@ -300,6 +300,9 @@
   </si>
   <si>
     <t>fixing some styles, putting first touches on Fledge Dictonary, About us write up</t>
+  </si>
+  <si>
+    <t>Added CMMC l2 controls to DB</t>
   </si>
 </sst>
 </file>
@@ -1879,10 +1882,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>5535</c:v>
+                  <c:v>5595</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3165</c:v>
+                  <c:v>3105</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11885,10 +11888,18 @@
       </c>
     </row>
     <row r="61" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C61" s="24"/>
-      <c r="D61" s="22"/>
-      <c r="E61" s="22"/>
-      <c r="F61" s="22"/>
+      <c r="C61" s="32">
+        <v>45977</v>
+      </c>
+      <c r="D61" s="22">
+        <v>60</v>
+      </c>
+      <c r="E61" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="F61" s="22" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="62" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C62" s="25"/>
@@ -17574,11 +17585,11 @@
       </c>
       <c r="D2">
         <f>SUM(Table2[Time (Mins)])</f>
-        <v>5535</v>
+        <v>5595</v>
       </c>
       <c r="E2">
         <f>8700-D2</f>
-        <v>3165</v>
+        <v>3105</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Start AC l2 and rework how assessment objectives are displayed
</commit_message>
<xml_diff>
--- a/02_WorkingDocs/CMMCFledge_Workbook.xlsx
+++ b/02_WorkingDocs/CMMCFledge_Workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ckm32\OneDrive\Desktop\CMMCFledge\02_WorkingDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91622F2E-6951-4B19-A271-7A4917CE2419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2D8BBBA-B9F6-4848-B56F-09D32F9DF043}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40290" yWindow="3735" windowWidth="23040" windowHeight="12120" activeTab="1" xr2:uid="{208106DA-3D21-4604-99AA-9AD5A5B6DE72}"/>
+    <workbookView xWindow="38280" yWindow="2325" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{208106DA-3D21-4604-99AA-9AD5A5B6DE72}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="91">
   <si>
     <t>Week:</t>
   </si>
@@ -311,6 +311,9 @@
   </si>
   <si>
     <t>Building out L2 assessment outline</t>
+  </si>
+  <si>
+    <t>Building out L2 assessment</t>
   </si>
 </sst>
 </file>
@@ -1890,10 +1893,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>6015</c:v>
+                  <c:v>6285</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2685</c:v>
+                  <c:v>2415</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11966,22 +11969,46 @@
       </c>
     </row>
     <row r="66" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C66" s="25"/>
-      <c r="D66" s="23"/>
-      <c r="E66" s="23"/>
-      <c r="F66" s="23"/>
+      <c r="C66" s="33">
+        <v>45981</v>
+      </c>
+      <c r="D66" s="23">
+        <v>45</v>
+      </c>
+      <c r="E66" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="F66" s="23" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="67" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C67" s="24"/>
-      <c r="D67" s="22"/>
-      <c r="E67" s="22"/>
-      <c r="F67" s="22"/>
+      <c r="C67" s="32">
+        <v>45982</v>
+      </c>
+      <c r="D67" s="22">
+        <v>75</v>
+      </c>
+      <c r="E67" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="F67" s="22" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="68" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C68" s="25"/>
-      <c r="D68" s="23"/>
-      <c r="E68" s="23"/>
-      <c r="F68" s="23"/>
+      <c r="C68" s="33">
+        <v>45679</v>
+      </c>
+      <c r="D68" s="23">
+        <v>150</v>
+      </c>
+      <c r="E68" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="F68" s="23" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="69" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C69" s="24"/>
@@ -17625,11 +17652,11 @@
       </c>
       <c r="D2">
         <f>SUM(Table2[Time (Mins)])</f>
-        <v>6015</v>
+        <v>6285</v>
       </c>
       <c r="E2">
         <f>8700-D2</f>
-        <v>2685</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
L2 AT result built
</commit_message>
<xml_diff>
--- a/02_WorkingDocs/CMMCFledge_Workbook.xlsx
+++ b/02_WorkingDocs/CMMCFledge_Workbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ckm32\OneDrive\Desktop\CMMCFledge\02_WorkingDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8844F5B6-4448-42CD-8426-8342A009F146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AC41099-2EF0-4BA1-B77F-D3EFE7A478AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="2325" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{208106DA-3D21-4604-99AA-9AD5A5B6DE72}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="93">
   <si>
     <t>Week:</t>
   </si>
@@ -317,6 +317,9 @@
   </si>
   <si>
     <t>Outside stakeholder discussion</t>
+  </si>
+  <si>
+    <t>Building out L2 assessment, AC/AT</t>
   </si>
 </sst>
 </file>
@@ -1896,10 +1899,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>6375</c:v>
+                  <c:v>6495</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2325</c:v>
+                  <c:v>2205</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12004,13 +12007,13 @@
         <v>45983</v>
       </c>
       <c r="D68" s="23">
-        <v>210</v>
+        <v>330</v>
       </c>
       <c r="E68" s="23" t="s">
         <v>27</v>
       </c>
       <c r="F68" s="23" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="69" spans="3:6" x14ac:dyDescent="0.3">
@@ -17663,11 +17666,11 @@
       </c>
       <c r="D2">
         <f>SUM(Table2[Time (Mins)])</f>
-        <v>6375</v>
+        <v>6495</v>
       </c>
       <c r="E2">
         <f>8700-D2</f>
-        <v>2325</v>
+        <v>2205</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">

</xml_diff>